<commit_message>
docs: cycle-damping campaign + fly-away root cause (skill + test records CB52-55)
tune-plasmc skill: 2026-06-20 addendum -- yaw cycle is the master driver (kOmega_z
root fix; check yaw first), fly-away = terminal 1/z positive-feedback launch (kappa
can't fix it, enters u_eq c-term), h_ez non-convergence, and the validate-across-seed-
ensemble methodology lesson.

test records CB52-55: chi_r/kR/kOmega_z bake; h_rd bake+revert (seed fragility);
fly-away 1/z mechanism trace; h_ez non-convergence.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MATLAB/test_data/MATLAB_test_record.xlsx
+++ b/MATLAB/test_data/MATLAB_test_record.xlsx
@@ -1626,7 +1626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F52"/>
+  <dimension ref="A1:F56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -3301,6 +3301,134 @@
         </is>
       </c>
     </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>CB52</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>cb_chi/kr/komz bake (VDF_ASMC clean blocks)</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>Cycle-damping gain campaign on the clean single controller. chi_r 0.85-&gt;1.15 (full +-40%); kR-roll 1.5-&gt;2.5 (Y-attitude damping); kOmega_z 0.1-&gt;0.2</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t>chi_r=1.15 (4b87e20): full +-40% guaranteed, keeps 25/25. kR=2.5 (c383a64): SHARP optimum (2.0 near-divergent, 4.0 collapse), damps Y-lateral cycle. kOmega_z=0.2 (783f462): the ROOT fix -- per-axis map found YAW cycle (Circ-IC3=1.78) PUMPS the lateral cycles via yaw&lt;-&gt;image coupling; 0.2 kills yaw -90% AND lateral (Y 0.98-&gt;0.11) MONOTONICALLY, zero gate cost. All bit-exact blocks-vs-canonical |delta|=0</t>
+        </is>
+      </c>
+      <c r="F53" s="4" t="inlineStr">
+        <is>
+          <t>kOmega_z (yaw rate damping) is the master cycle lever -- CHECK YAW FIRST on any lateral-cycle problem. kR=2.5 sharp = robustness risk. Per-axis cycle map: Z-descent 0.48 now largest (irreducible)</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>CB53</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>cb_hrd floor + revert (60ac526-&gt;593f0d6)</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>h_rd 0.42-&gt;0.40 to shrink the descent cycle (deep sweep flagged h_rd as the only lever moving the descent floor)</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>h_rd=-0.40 shrinks descent cycle -21% (0.48-&gt;0.375), CLEAN on seeds 1,2,3 (real 25/25). BUT comparison regen (seed 1002) exposed catastrophic fly-aways (vel 33!). Reverting h_rd-&gt;-0.42 fixed seed1002 (5/5) + broad robustness 51/55 vs 46/55. Gentler/slower descent spends MORE time in low-alt 1/z danger zone -&gt; more fly-aways</t>
+        </is>
+      </c>
+      <c r="F54" s="4" t="inlineStr">
+        <is>
+          <t>h_rd=-0.42 STANDS. Smaller cycle != more robust. LESSON: validate gains across a SEED ENSEMBLE, not seed1+noiseless -- the campaign shipped a fragile h_rd by optimizing on seed1</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>CB54</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>cb_flyaway/fa2/spike2 (trace)</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>WHY does the quadrotor fly away? Trace Linear-IC2 seed1004 (vel 23.7)</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>NOT a slow drift, NOT a noise outlier. Drone descends CLEANLY 31s to alt 0.33m (0.13m above zf=0.20), then LAUNCHES upward (alt 0.33-&gt;16m, descVz=-22.79). dPdt ramps GRADUALLY 161-&gt;472 (not a discrete jump); baseline dPdt~200 at 0.35m = 7x noise floor (geometry not noise). V_h(3) ramps WHILE altitude reverses = POSITIVE FEEDBACK. Root = terminal 1/z geometric instability: loom V_h(3)=vz/z has loop gain proportional 1/z-&gt;inf near touchdown; self-excites (V_h(3)up-&gt;thrust-&gt;ascent-&gt;dPdt up-&gt;V_h(3) up). Noise SEEDS it, geometry provides the gain; a race descent-to-zf vs loop igniting</t>
+        </is>
+      </c>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t>FLY-AWAY = terminal 1/z positive-feedback launch, a PERCEPTION-FRONT-END limit (same 1/z wall as lateral precision). Explains seed-dependence + the h_rd paradox (gentler=more danger-zone time). Fix = bound V_h(3) or fix the regulation</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>CB55</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>cb_hez (h_ez convergence)</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>User insight: regulating the loom should make d(area)/dt constant (dPdt flat, not ramping). Is h_ez=V_h_e(3) converging to 0?</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>NO. V_h_d(3)=-0.42 (correct, constant) but V_h(3) only reaches ~-0.3 -&gt; persistent h_ez ~+0.12 in BOTH clean AND fly-away. The descent loom is regulated to ~-0.3, NOT commanded h_rd=-0.42 -&gt; loom NOT constant -&gt; area rate NOT constant -&gt; dPdt RAMPS -&gt; enables the 1/z instability. Root = weak descent integral (chi_z=0.025 + izeta2_max=5 clamp -&gt; max authority ~0.125, can't null steady-state loom error). kappa CAN'T help: 1/z spike enters u_eq c-term -h_z*h (quadratic), bypasses u_sw/kappa; kappa assumes sigma correctly measured (this is sensor-side)</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>h_ez non-convergence is the ROOT regulation defect behind the fly-away. PROPER fix = strengthen descent integral so h_ez-&gt;0 (constant loom = constant area rate = scale-free soft touchdown); band-aid = LOOM_CLAMP V_h(3) before SG filter (gated, default-off). Descent-integral (chi_z/izeta) strengthening prototype in progress</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
docs+figures: aggressive-baseline regen + session findings (CB56-60)
- Regenerated multi-init + multi-speed figures at the committed aggressive baselines
  (Linear 1.1x, Sin 1.67x, Liss reshaped+2.125x, Circ 1.6x): multi-init 25/25,
  multi-speed full ±40%. (Comparison deferred — baseline controllers being retuned.)
- tune-plasmc skill: 2026-06-21 addendum (chi_z=0.1/E_z=0.5 bakes; the two fundamental
  limits = visibility-CBF lateral ceiling + ±90° yaw alias; aggressive-target methodology).
- Test records CB56-60 (chi_z, E_z, lateral/yaw limit audits, aggressive baselines).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MATLAB/test_data/MATLAB_test_record.xlsx
+++ b/MATLAB/test_data/MATLAB_test_record.xlsx
@@ -1626,7 +1626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F56"/>
+  <dimension ref="A1:F61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -3429,6 +3429,166 @@
         </is>
       </c>
     </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>CB56</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>cb_chi_z bake (67ab71f)</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>Strengthen descent integral so h_ez-&gt;0: bake chi_z 0.025-&gt;0.1. Does it kill the 1/z fly-away?</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="inlineStr">
+        <is>
+          <t>YES. chi_z=0.1: |h_ez| S1-&gt;0.107, fly-aways 35-&gt;3/300 (-91%), SP 87-&gt;97%, full gate, bit-exact. chi_z=0.2+Gamma_z=1.0 REJECTED: BETTER h_ez (0.103) but WORSE robustness (NL 25-&gt;24, fly 3-&gt;13) -- past 0.1 more loop gain OVER-DRIVES the cascade lag. h_ez-convergence and fly-away robustness DIVERGE past chi_z=0.1. The 3 residual fly = Static-IC5 mid-descent FALSE h_ez convergence (loom UNDER-reports the fast descent: measured -0.34 vs true -0.78 -&gt; h_ez looks +0.08 while truly overshooting vz 1.27 vs cmd 0.68 -&gt; sign-flip -&gt; launch)</t>
+        </is>
+      </c>
+      <c r="F57" s="2" t="inlineStr">
+        <is>
+          <t>chi_z=0.1 = descent optimum (the integral GAIN matters, not the izeta clamp). Superseded the LOOM_CLAMP band-aid (reverted). 3 residual = Static-IC5 perception front-end limit, not gain-tunable</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>CB57</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>cb_ez/sigz/chat/pz bake (aeb4283)</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>User: kappa IS the damping. Why isnt it damping the Z limit cycle? Can E_z engage it?</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>The Z cycle rings 100% INSIDE the boundary layer (|sigma_z|/E_z&lt;=0.2 -&gt; sat linearized -&gt; kappa switching LOCKED OUT) AND kappa_z is leaked down (0.25-&gt;0.15). E_z 1.0-&gt;0.5 engages the switching -&gt; Z cycle -8% (0.63-&gt;0.58) + better h_ez, full gate, bit-exact. E_z&lt;0.5 hard-switch OVER-DRIVES the aggressive cells (NL 25-&gt;20, fly 14; sigma_z NOISE is only 0.05 -&gt; NOT noise chatter, it is sat-saturation on large-sigma_z offset cells S3/S5/L3/C5). P_z=20 (smaller kappa) recovers 4/5 broken cells but trades damping. X/Y cycles ALSO 100% inside the layer BUT tightening E_x/E_y makes them WORSE (X 0.34-&gt;0.42) -- they are NOISE-PUMPED (s_ddot positive feedback) so kappa switching FEEDS them</t>
+        </is>
+      </c>
+      <c r="F58" s="4" t="inlineStr">
+        <is>
+          <t>E_z=0.5 baked (sweet spot). Z=under-damped (kappa helps via E_z), X/Y=forced/noise-pumped (kappa hurts; s_ddot-drop is the lever). DIFFERENT mechanisms -- dont apply the E_z fix to lateral</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>CB58</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>cb_latlim/aggrtune/aggr3 (lateral-limit audit)</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>Does the test run hit any LIMIT in lateral control on a fast/offset target (Linear-IC3 @2x)? Retune chi_r/Gamma to catch faster targets?</t>
+        </is>
+      </c>
+      <c r="E59" s="2" t="inlineStr">
+        <is>
+          <t>The VISIBILITY-CBF is the limit, NOT the gains. CBF cuts commanded lateral accel to 9% of demand (100% of steps), lean 100% CONE-clamped (theta_cone not the 60deg cap), position-funnel-y rails 22%. The flow funnel S_2 is NOT saturated (0.05) -&gt; control GAINS have headroom, bottleneck is DOWNSTREAM. chi_r=2 REGRESSES the nominal set 24-&gt;18; chi_r2+cone-relax only gets xy 4.75-&gt;2.93 STILL FoV-breaching. fov_inset/theta_cap zero effect (marker leaves AHEAD because drone falls behind, not over-lean)</t>
+        </is>
+      </c>
+      <c r="F59" s="2" t="inlineStr">
+        <is>
+          <t>Lateral ceiling = the target-visibility CBF (the papers own guarantee) = visibility-vs-agility tradeoff hard-capped by camera FoV. NOT gain-tunable. Fix = wider FoV (hardware) or anticipatory guidance. AUDIT THE LIMITS before retuning -- gains usually have headroom</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>CB59</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>cb_yawlim/yawconv (yaw-limit audit)</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>Does the test run hit a LIMIT in yaw control (Circular wz=1.0, yaw err blew to 40deg)? Increase e_a convergence to fix?</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="inlineStr">
+        <is>
+          <t>Yaw limit = +-90deg MARKER-SYMMETRY ALIAS (virtual-compass observability). e_a hits 89.8deg (IC4) right at the unwrap edge; square marker observable only to +-90deg. The yaw ASMC switching is NOT saturated (sat max 0.89, kappa_a healthy) -&gt; gains have headroom. Inner loop yaw-rate lags (cmd 2.85 vs achieved 1.62). Faster e_a convergence (kappa_a0=5/Gamma_a=2) DOES pull e_a off the alias (89.8-&gt;49deg) BUT cant rescue wz=1.0 (lateral FoV co-binds); at wz=0.75 lateral breaches with yaw still fine (&lt;=21deg) -&gt; yaw boost is MOOT. Yaw only binds AFTER the lateral collapse drags the drone far behind</t>
+        </is>
+      </c>
+      <c r="F60" s="2" t="inlineStr">
+        <is>
+          <t>Yaw ceiling = +-90deg observability (perception, like lateral), NOT gains. Coupled to lateral FoV failure. e_a-convergence boost real but cannot extend a lateral-bound case. At Circ wz=0.5 (clean ceiling) yaw err=2.9deg, full margin</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>CB60</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>traj_Gen aggressive baselines + cb_*sweep/finalval (UNCOMMITTED + REGEN PENDING)</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="inlineStr">
+        <is>
+          <t>Make moving-target trajectories more aggressive while keeping 25/25 + +-40%</t>
+        </is>
+      </c>
+      <c r="E61" s="2" t="inlineStr">
+        <is>
+          <t>LOCKED set (5-IC 25/25 + centered +-40%, both seeds; committed 90ef528): Linear 1.1x, Sinusoidal v0=0.5 (1.67x), Lissajous w1 -0.8-&gt;-0.5 (reshaped) + w2 0.4-&gt;0.85, Circular wz=0.4 (1.6x). TWO-TEST CONVENTION (was conflated): 25/25 = 5-IC set at baseline (offset ICs bind); +-40% = CENTERED-IC speed sweep (2-3x more headroom). 5-IC ceilings: Linear 1.1x (visibility-CBF floor), Sin ~1.9x, Liss 2.5x (+25% collapses), Circ 2.0x (wz=1.0 -&gt; 0/10 on BOTH lateral FoV AND +-90 yaw alias). Linear edit-bug caught: v=2.0 with p=1.0 -&gt; v!=dp/dt corrupts rel-vel check (verify p,v same multiplier)</t>
+        </is>
+      </c>
+      <c r="F61" s="2" t="inlineStr">
+        <is>
+          <t>Substantially more aggressive (Liss 2.1x, Circ 1.6x, Sin 1.67x) keeping both guarantees. Linear is the floor (visibility-CBF catch-up). OPEN: +-40% centered-vs-5-IC convention. PENDING: commit traj_Gen + full dataset/figure REGEN (stale at old baselines)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
records+memory: 2026-06-26..07-02 MATLAB campaign — LOCKED kappa-engaged bake, yaw observability (2pi port, ~0.5 rad/s architectural ceiling), prescribed-rate h_d (OPEN: missing S_r_dot term); test record F17-F21 + locked_yaw_hd_log; sync-gains skill vdf_params addendum
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MATLAB/test_data/MATLAB_test_record.xlsx
+++ b/MATLAB/test_data/MATLAB_test_record.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="cthilde_test_log" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="findings" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="combined_barrier_log" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cthilde_test_log" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="findings" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="combined_barrier_log" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="locked_yaw_hd_log" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1320,7 +1321,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:D22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1700,6 +1701,116 @@
       <c r="D17" s="2" t="inlineStr">
         <is>
           <t>Quantifies the pre-combined-barrier SEN-funnel baseline the authority analysis was run against</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>F17</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>LOCKED kappa-engaged config baked in vdf_params.m (kappa0 .05 / N .10 / Pleak [.5;.5;1.5] / E .5 / Xi_r .3 / p_rinf .85 / theta_per_axis): 25/25 SP gate + 7x-stress 5/5 (vs 3/5 old baked) + kappa_z adapts MONOTONE 5.6x RMS (.057-&gt;.318) / 7.2x peak over the {0,1,3,5,7}x stress ladder. E gates switching DELIVERY not adaptation; E_xy=0.5 floor (lower pumps terminal velocity); p_h untightenable (funnel overtakes h_e); p_rinf floor ~0.85 (engR-&gt;1 below).</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>LK1-LK9 (locked_yaw_hd_log sheet); MATLAB/Datasets/MultiInit/kappa_adapt.mat; memory Memory/matlab/project_locked_kappa_engagement</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Funnels+kappa now ENGAGED -&gt; real disturbance margin for Gazebo; p_rinf=0.85&lt;1 needs Standing-Cond-1 manuscript framing</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>F18</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Yaw +-90deg observability ceiling: alpha = 0.5*atan2(2mu11, mu20-mu02) uses only EVEN-order (2nd) moments -&gt; invariant under 180deg -&gt; orientation observable mod 180 only; yaw_asmc's x2../2 unwrap folds e_a to +-90 and fast heading swings PIN e_a at 90 (no gain can act on unrepresentable error -- e_a stays 88-90deg across EVERY yaw param). FIX = PX4-parity weighted 2pi port (corner weights [4,3,2,1], weighted-centroid displacement = odd 1st moment disambiguates the pi-axis); verified clean 360 sweep; unwrap removed; gate 25/25.</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Y1-Y7 (locked_yaw_hd_log); Obsolete/image_feature_pre_weighted2pi.m; memory Memory/matlab/project_yaw_observability_campaign</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>MATLAB perception now matches PX4 _marker_principal_angle; yaw error is a faithful +-180 signal</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>F19</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Yaw-rate ceiling ~0.5 rad/s is ARCHITECTURAL, not gain-tunable: at 2x Circular yaw (0.96 rad/s) the failure is LATERAL (termEa only 14-18deg) -- s_e expressed in the drone-yaw-aligned V frame ORBITS at the yaw rate; radial convergence must ride on top of orbit-tracking and the accel budget saturates (CBF cone-sat frac 0.66-&gt;0.86) until the position funnel breaches (engR 1.16). chi_r 2-&gt;4 no help; kR_yaw=1.0 marginal (2/5, breaks oscillating-heading cases); yaw-rate FF Omega_d=u_a REVERTED (u_a is the lagged output -- circular).</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Y5-Y6, Y9 (locked_yaw_hd_log); cone-sat/engR vs yaw-mult audit</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Levers = wider accel budget or yaw-fixed lateral frame (research scope); manuscript range 0.29-0.67 rad/s sits inside the ceiling</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>F20</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Heading-yaw (tangent atan2(vy,vx)) on Sin/Liss: Sinusoidal trackable post-2pi with gentle Gamma_a=0.15 (5/5 realistic + speed; its vy=v0&gt;0 bounds the swing); Lissajous INTRACTABLE -- velocity ~vanishes at reversals (A=0.4: max|psi_dot|=32 rad/s) -&gt; ~180 snaps; rate-limited stateful heading does NOT fix (Sin regresses 4/5, Liss 1/5); larger A softens (worstXY 39-&gt;5) but 0/5 at all A. REVERTED -- traj_Gen restored (Sin/Liss non-rotating); Circular remains the yaw-exercising case (kappa_a adapts to sigma_a~0.95 -&gt; ~0.5 equilibrium).</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Y1-Y4, Y8, Y10 (locked_yaw_hd_log)</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>A non-rotating Liss target is the physically honest model; heading-yaw enablement parked, revertible from Obsolete/</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>F21</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Prescribed-rate h_d (user design): h_d xy term s_dot_meas -&gt; phi_max.*S_r.*dp_r; derivative is 1000x smaller (RMS .007 vs measured s_ddot ~7) -&gt; folded into dh_d/c-term, s_ddot-drop REMOVED. Gate 25/25+25/25 noiseless, speed 20/20; A/B: standard stress equivalent (no breach occurs), BREACHING scenario (2x yaw) prescribed engR 0.76 NO-breach vs measured 1.16 breach. OPEN: formula incomplete -- s_e=phi_max*S_r*p_r =&gt; full deriv needs phi_max*(S_r_dot*p_r + S_r*dp_r); current form assumes S_r_dot=0; awaiting prescribed S_r_dot contraction law.</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Y11-Y13 (locked_yaw_hd_log); Obsolete/{position_funnel,flow_surface}_pre_prescrate.m; memory Memory/matlab/project_prescribed_rate_hd</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Bounded-on-breach h_d = recovery authority (validated); DO NOT commit/port to PX4 until the S_r_dot term is resolved</t>
         </is>
       </c>
     </row>
@@ -3680,4 +3791,794 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F24"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="7" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="62" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Trial</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Harness (cb_*.m)</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>What varied</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Result</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Verdict</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>LK1</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>cb_engage_probe/sweep</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>nominal engagement audit on old baked config</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>funnel/kappa IDLE in nominal (engR~0.6 only at IC5); no margin for real disturbance</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>retune needed</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>LK2</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>cb_D_fulltest</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>config D (kappa0 .05, N .10, Pleak [.5;.5;1.5]) 5 traj x 5 IC</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>25/25 SP realistic; kappa active</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>D holds the gate</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>LK3</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>cb_kappa_reject</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>D vs old-baked under stress escalation per axis</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>kappa adapts UP under stress (kRMS_xy .07-&gt;.19) where baked stays flat; 7x stress 5/5 vs baked 3/5</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>kappa DEMONSTRABLY rejects; 7x margin</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>LK4</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>cb_E_kappa_sigma/E25_validate</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>boundary layer E_xy {0.25,0.5,1.0}</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>wide E_x=1.0 gates lateral switching (delivery); E_xy&lt;0.5 pumps terminal velocity</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>E=0.5 floor; E gates delivery NOT adaptation</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>LK5</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>cb_kappa_validate/threshold</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>KNOWN_DIST hook: Fx=3N step on [2,6]s (Static)</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>kappa_x rises +43% while force on, leak-decays after off</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>adaptation law verified against known input</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>LK6</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>cb_funnel_tighten/imgfunnel/lock_ph</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Xi_r .10-&gt;.3 + p_rinf 1.0-&gt;.85; then p_h tighten</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>pr-tight: xy .013-&gt;.011 (~15%), 25/25 held; p_h tighten FAILS (funnel overtakes h_e convergence, 14/25)</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>bake pr-tight; p_h untightenable</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>LK7</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>cb_lock_fulltest</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>LOCKED (D + E.5 + pr-tight) full manuscript battery</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>25/25 gate + speed 40/40 (+-40%) + multi-init 50/50 + comparison Proposed SP all</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>LOCKED baked into vdf_params</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>LK8</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>cb_pr_reduce</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>p_rinf {0.85,0.70,0.60,0.50} below the bake</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>lower p_rinf -&gt; maxEngR climbs toward 1 (breach margin gone); no precision gain worth it</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>0.85 = floor</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>LK9</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>cb_lock_kappa/cb_kappa_adapt_data</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>kappa vs disturbance ladder {0,1,3,5,7}x, 10 cells</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>kappa_z RMS .057/.073/.137/.220/.318 MONOTONE (5.6x); peak 7.2x; x 2.7x, y 1.7x (peak)</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>genuine adaptation; kappa_adapt.mat</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>LK10</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>cb_gamma_why/cb_au_decomp</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>why Gamma can't replace kappa (terminal balloon mechanics)</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>switching term theta*sat*kappa = 94% of terminal a_u spike; reaching a_u 47.3 @Gamma=2 vs 10.4 baked (G_2^-1 amplification)</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>Gamma over-drives; kappa is the right lever</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Y1</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>(traj_Gen heading yaw)</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>tangent heading atan2(vy,vx) on Sin/Liss</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Sin: realistic 5/5, speed 5/5, noiseless 4/5; Liss: 0/3 fly-away (~180deg heading snaps)</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>Sin near-works; Liss pathological</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Y2</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>cb_yawret</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>yaw-gain screen on Sin noiseless failure</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>gentler recovers (Gamma_a .15 -&gt; 5/5, E_a 8 -&gt; 5/5); faster (Gamma_a .5, Omega_a .5) -&gt; 3/5</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>failure = yaw-&gt;lateral PUMP, not lag</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Y3</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>cb_yawlag/cb_yawlc</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>trace target/drone yaw + limit-cycle check</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>drone swings 140deg vs target 77deg (~90deg phase lag, overshoot); sat(sigma_a/E_a) frac 0.00, rate flips 4-6</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>bandwidth-limited FORCED track; NO limit cycle</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Y4</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>cb_eaconv</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>e_a convergence per 2s window</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>amplitude steady 20-90deg ALL windows to touchdown; peaks pinned at 90deg</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>bounded NOT converging; 90deg = observability ceiling</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Y5</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>cb_kryaw/cb_yawall</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>kR_yaw {0.5-2.5}, kOmega_yaw {0.1-0.6}, all ASMC levers</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>e_a stays 88-90deg at EVERY setting; kR_yaw&gt;=1 breaks Sin (3/5); kOmega_yaw pinned 0.2 (down=cycle, up=lag)</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>NO gain reduces the lag; inner levers exhausted</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Y6</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>(so3_tracker yaw FF)</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Omega_d=[0;0;u_a] feedforward</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>Circular helped (e_a 53deg, 5/5); Sin 5/5-&gt;3/5 (u_a = lagged output, FF amplifies the swing)</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>REVERTED; circular feedback</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Y7</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>cb_rotsweep + gate</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>2pi weighted-corner orientation port (PX4 parity) + unwrap removal</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>synthetic 360 sweep CLEAN (15deg steps, no fold); full gate 25/25 realistic + 25/25 noiseless; alpha_d auto-correct (Static termEa -0.0deg)</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>2pi orientation KEPT (uncommitted)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Y8</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>cb_yawtune/cb_yawterm</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>post-2pi gentle retune + terminal-lag levers</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>Ga.15/Oa.15/Ea6 all recover Sin heading-yaw 5/5; Omega_a=0.4 cuts Circ termEa 17-&gt;9deg but Sin 41-&gt;60deg (windup on oscillating ref)</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
+          <t>gentle linear yaw wins; integral only for constant yaw</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Y9</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>cb_circyaw/cb_coupling/cb_caps/cb_chitest/cb_kryaw2</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Circular yaw-rate mult {1,2,3,4,6}x + cap audit</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>1x 5/5 -&gt; 2x 1/5 -&gt; 3x+ 0/5; s_e ORBITS at yaw rate; cone-sat frac .66/.71/.86; funnel breach engR 1.16 @2x; chi_r 2-4 flat; kR_yaw1.0 2/5</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>~0.5 rad/s ceiling ARCHITECTURAL (frame coupling + accel budget)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Y10</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>cb_wmax/cb_lissA*/cb_relax</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>rate-limited stateful heading (w_max .05-.4) + Liss A/freq relax</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>rate-limit does NOT fix (Sin 4/5 all w_max; Liss 1/5); bigger A softens raw-heading severity (worstXY 39-&gt;5) but 0/5</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>REVERTED -- traj_Gen restored; Liss stays non-rotating</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Y11</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>cb_dhd/cb_presc/cb_fold/cb_sinliss</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>prescribed-rate h_d: s_dot_meas -&gt; phi_max.*S_r.*dp_r, then folded into dh_d</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>d(s_dot_presc)/dt RMS .007 vs measured s_ddot ~7 (1000x smaller) -&gt; s_ddot-drop removed; gate 25/25 + 25/25 noiseless (baked gains)</t>
+        </is>
+      </c>
+      <c r="F22" s="4" t="inlineStr">
+        <is>
+          <t>smooth + consistent h_d/dh_d; validated</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Y12</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>cb_ab/cb_ab2</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>A/B prescribed vs measured h_d, same seeds</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>standard stress 1-7x EQUIVALENT (5/5 both, engR .59, no breach); BREACHING 2x-yaw: prescribed engR .76 NO-breach + worstXY 1.12 vs measured 1.16 breach + 1.56; speed sweep 20/20</t>
+        </is>
+      </c>
+      <c r="F23" s="4" t="inlineStr">
+        <is>
+          <t>bounded-on-breach benefit CONFIRMED</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Y13</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>(user review)</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>formula audit of s_dot_presc</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>phi_max.*S_r.*dp_r assumes S_r CONSTANT; s_e=phi_max*S_r*p_r =&gt; missing phi_max*S_r_dot*p_r term; measured S_r_dot would collapse to s_dot_meas (circular)</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>OPEN -- awaiting prescribed S_r_dot contraction law</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
records: PX4 GT-FB bake cross-port A/B on MATLAB gate — REJECTED (Gamma_xy .25 reaching-starved, Xi_h fast-contraction kills 7x margin); divergences stand documented (row P1, cb_px4port.m)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MATLAB/test_data/MATLAB_test_record.xlsx
+++ b/MATLAB/test_data/MATLAB_test_record.xlsx
@@ -3799,7 +3799,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F24"/>
+  <dimension ref="A1:F25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -4578,6 +4578,38 @@
         </is>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>cb_px4port</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>PX4 GT-FB bakes on the MATLAB gate: Gamma_xy=0.25, Xi_h=[0.7,0.7,1.0], both (vs baked LOCKED)</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>baked 25/25 (mXY .011, 7x 5/5); Gxy.25 23/25 worstXY 2.63 (reaching-starved in engaged-funnel design); Xih 22/25 + 7x 1/5 (p_h-overtake via contraction rate); both 19/25 + 7x 0/5. Already-converged: N=.10, P2INF_xy=1.0, cbf2-only, no backstepping h_d</t>
+        </is>
+      </c>
+      <c r="F25" s="4" t="inlineStr">
+        <is>
+          <t>PX4 bakes REJECTED on MATLAB -- regime-specific (wide-funnel PR0=10 vs engaged p_r0=1.2); divergences stand documented</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
records: prescribed-rate h_d RESOLVED — formula complete as definition (h_e = p_10*zeta_r_dot/g_r; S_r_dot law rejected as wrong approach; finite-diff dh_d kept); row Y14, F21 updated
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MATLAB/test_data/MATLAB_test_record.xlsx
+++ b/MATLAB/test_data/MATLAB_test_record.xlsx
@@ -1800,17 +1800,17 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Prescribed-rate h_d (user design): h_d xy term s_dot_meas -&gt; phi_max.*S_r.*dp_r; derivative is 1000x smaller (RMS .007 vs measured s_ddot ~7) -&gt; folded into dh_d/c-term, s_ddot-drop REMOVED. Gate 25/25+25/25 noiseless, speed 20/20; A/B: standard stress equivalent (no breach occurs), BREACHING scenario (2x yaw) prescribed engR 0.76 NO-breach vs measured 1.16 breach. OPEN: formula incomplete -- s_e=phi_max*S_r*p_r =&gt; full deriv needs phi_max*(S_r_dot*p_r + S_r*dp_r); current form assumes S_r_dot=0; awaiting prescribed S_r_dot contraction law.</t>
+          <t>Prescribed-rate h_d (user design): h_d xy term s_dot_meas -&gt; phi_max.*S_r.*dp_r; derivative is 1000x smaller (RMS .007 vs measured s_ddot ~7) -&gt; folded into dh_d/c-term, s_ddot-drop REMOVED. Gate 25/25+25/25 noiseless, speed 20/20; A/B: standard stress equivalent (no breach occurs), BREACHING scenario (2x yaw) prescribed engR 0.76 NO-breach vs measured 1.16 breach. RESOLVED (Y14): formula complete as a DEFINITION -- h_e,xy = p_10*zeta_r_dot/g_r (S_r varying IS the signal; S_r_dot law rejected as wrong approach); finite-diff dh_d kept per user.</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Y11-Y13 (locked_yaw_hd_log); Obsolete/{position_funnel,flow_surface}_pre_prescrate.m; memory Memory/matlab/project_prescribed_rate_hd</t>
+          <t>Y11-Y14 (locked_yaw_hd_log); Obsolete/{position_funnel,flow_surface}_pre_prescrate.m; memory Memory/matlab/project_prescribed_rate_hd</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Bounded-on-breach h_d = recovery authority (validated); DO NOT commit/port to PX4 until the S_r_dot term is resolved</t>
+          <t>Bounded-on-breach h_d = recovery authority (validated); MATLAB form final (016855e); PX4 port = separate decision</t>
         </is>
       </c>
     </row>
@@ -3799,7 +3799,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F25"/>
+  <dimension ref="A1:F26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -4574,37 +4574,69 @@
       </c>
       <c r="F24" s="3" t="inlineStr">
         <is>
-          <t>OPEN -- awaiting prescribed S_r_dot contraction law</t>
+          <t>OPEN -- S_r_dot question raised</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
+          <t>Y14</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>(user resolution)</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>S_r_dot contraction law proposal REJECTED by user (wrong approach)</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>correct reading: h_d = p_10*S_r*p_r_dot is the funnel-consistent reference by DEFINITION; S_r varying is the SIGNAL -- h_e,xy = sdot - p_10*S_r*p_r_dot = p_10*zeta_r_dot/g_r (barrier-coordinate rate; sigma = true PD pair on zeta_r). A prescribed S_r_dot would make the reference the convergence driver (violates funnel-as-constraint). dh_d: finite-diff kept per user (tiny S_r_dot content RMS .007, gate-validated) over analytic S_r-frozen</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>RESOLVED -- formula complete; code final at 016855e</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="B25" s="2" t="inlineStr">
+      <c r="B26" s="2" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="C25" s="2" t="inlineStr">
+      <c r="C26" s="2" t="inlineStr">
         <is>
           <t>cb_px4port</t>
         </is>
       </c>
-      <c r="D25" s="2" t="inlineStr">
+      <c r="D26" s="2" t="inlineStr">
         <is>
           <t>PX4 GT-FB bakes on the MATLAB gate: Gamma_xy=0.25, Xi_h=[0.7,0.7,1.0], both (vs baked LOCKED)</t>
         </is>
       </c>
-      <c r="E25" s="2" t="inlineStr">
+      <c r="E26" s="2" t="inlineStr">
         <is>
           <t>baked 25/25 (mXY .011, 7x 5/5); Gxy.25 23/25 worstXY 2.63 (reaching-starved in engaged-funnel design); Xih 22/25 + 7x 1/5 (p_h-overtake via contraction rate); both 19/25 + 7x 0/5. Already-converged: N=.10, P2INF_xy=1.0, cbf2-only, no backstepping h_d</t>
         </is>
       </c>
-      <c r="F25" s="4" t="inlineStr">
+      <c r="F26" s="4" t="inlineStr">
         <is>
           <t>PX4 bakes REJECTED on MATLAB -- regime-specific (wide-funnel PR0=10 vs engaged p_r0=1.2); divergences stand documented</t>
         </is>

</xml_diff>